<commit_message>
Web: cot 7 NLS chon loc du 35 tuan (ban 162)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CH3DVFLNt2eFwxeEQw5xK2
</commit_message>
<xml_diff>
--- a/assets/docs/lop1/Dao duc - Lop 1.xlsx
+++ b/assets/docs/lop1/Dao duc - Lop 1.xlsx
@@ -627,7 +627,8 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>NLS-KT (Cơ bản 1): Chiếu phóng to tranh Khám phá của bài “Em tắm, gội sạch sẽ” cho HS so sánh hai bạn trong tranh.</t>
+          <t>Năng lực số Miền 1 (Cơ bản, bậc 1): GV chiếu phóng to tranh Khám phá của bài “Em tắm, gội sạch sẽ” cho HS so sánh hai bạn trong tranh
+Năng lực số Miền 5 (Cơ bản, bậc 1): GV mở bài tập tương tác kéo các bước tắm, gội về đúng thứ tự; máy báo đúng, sai ngay nên HS tự nhận ra chỗ xếp nhầm và sắp lại</t>
         </is>
       </c>
     </row>
@@ -661,7 +662,8 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>NLS-GQVĐ (Cơ bản 1): Mở bài tập tương tác sắp các bước mặc áo và chỉnh trang phục theo đúng thứ tự.
+          <t>Năng lực số Miền 1 (Cơ bản, bậc 1): GV chiếu phóng to tranh Khám phá của bài “Em giữ trang phục gọn gàng, sạch sẽ” và thêm vài ảnh thật: áo bỏ trong quần, cổ áo lật ngay ngắn
+Năng lực số Miền 5 (Cơ bản, bậc 1): GV mở bài tập tương tác sắp các bước mặc áo và chỉnh trang phục theo đúng thứ tự: mặc áo, cài cúc từ dưới lên, bỏ áo vào quần, chỉnh cổ áo
 KNS: KN tự phục vụ: tự làm lấy việc của mình, giữ gìn vệ sinh cá nhân và nơi ở.</t>
         </is>
       </c>
@@ -1039,7 +1041,8 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>NLS-GQVĐ (Cơ bản 1): Ở hoạt động Luyện tập, GV mở trên máy chiếu bài tập kéo thả.
+          <t>Năng lực số Miền 1 (Cơ bản, bậc 1): Ở hoạt động Khám phá bài “Giữ gìn tài sản của trường, lớp”, GV chiếu lên màn hình bộ ảnh chụp ngay tại trường mình: bộ bàn ghế còn lành và bộ bàn bị…
+Năng lực số Miền 5 (Cơ bản, bậc 1): Ở hoạt động Luyện tập, GV mở trên máy chiếu bài tập kéo thả: các bức tranh việc làm hiện ra, HS lên bảng kéo tranh vào cột “Nên làm” hoặc “Không nên làm”
 KNS: KN chi tiêu và giữ gìn: dùng đồ dùng, tiền bạc hợp lí, giữ gìn của công.</t>
         </is>
       </c>
@@ -1074,7 +1077,8 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>NLS-KT (Cơ bản 1): Ở hoạt động Khám phá bài “Giữ vệ sinh trường, lớp”, GV chiếu ảnh chụp chính lớp mình lúc đầu buổi và.
+          <t>Năng lực số Miền 1 (Cơ bản, bậc 1): Ở hoạt động Khám phá bài “Giữ vệ sinh trường, lớp”, GV chiếu ảnh chụp chính lớp mình lúc đầu buổi và sau khi trực nhật, phóng to góc để chổi
+Năng lực số Miền 5 (Cơ bản, bậc 1): Ở hoạt động Luyện tập, GV mở bài tập tương tác phân loại rác trên máy chiếu: máy hiện lần lượt vỏ hộp sữa, giấy vụn, lá cây
 KNS: KN tự phục vụ: tự làm lấy việc của mình, giữ gìn vệ sinh cá nhân và nơi ở.</t>
         </is>
       </c>
@@ -1109,7 +1113,8 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>NLS-GQVĐ (Cơ bản 1): Ở hoạt động Luyện tập, GV mở bài tập tương tác sắp xếp đồ dùng.
+          <t>Năng lực số Miền 1 (Cơ bản, bậc 1): Ở hoạt động Khám phá bài “Gọn gàng, ngăn nắp”, GV chiếu hai ảnh chụp cùng một góc học tập: lúc sách vở để lộn xộn và lúc đã xếp gọn
+Năng lực số Miền 5 (Cơ bản, bậc 1): Ở hoạt động Luyện tập, GV mở bài tập tương tác sắp xếp đồ dùng: máy hiện bàn học bừa bộn, HS kéo từng thứ về đúng chỗ là giá sách, hộp bút
 KNS: KN tự phục vụ: tự làm lấy việc của mình, giữ gìn vệ sinh cá nhân và nơi ở.</t>
         </is>
       </c>
@@ -1248,7 +1253,8 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>NLS-KT (Cơ bản 1): Ở hoạt động Khám phá bài “Tự giác tham gia các hoạt động ở trường”, GV chiếu ảnh chụp chính các hoạt động của trường mình.
+          <t>Năng lực số Miền 1 (Cơ bản, bậc 1): Ở hoạt động Khám phá bài “Tự giác tham gia các hoạt động ở trường”, GV chiếu ảnh chụp chính các hoạt động của trường mình: kế hoạch nhỏ, chăm sóc bồn hoa
+Năng lực số Miền 5 (Cơ bản, bậc 1): Ở hoạt động Luyện tập, GV mở bài tập tương tác: máy hiện các việc chung ở trường, HS chọn việc vừa sức mình có thể tự giác làm rồi bấm kiểm tra
 KNS: KN tự phục vụ: tự làm lấy việc của mình, giữ gìn vệ sinh cá nhân và nơi ở.</t>
         </is>
       </c>
@@ -1283,7 +1289,8 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>NLS-GQVĐ (Cơ bản 1): Ở hoạt động Luyện tập, GV mở bài tập tương tác phân loại.
+          <t>Năng lực số Miền 1 (Cơ bản, bậc 1): Ở hoạt động Khám phá bài “Tự giác làm việc nhà”, GV chiếu bộ ảnh những việc nhà vừa sức với HS lớp 1: gấp quần áo, tưới cây, nhặt rau, xếp dép
+Năng lực số Miền 5 (Cơ bản, bậc 1): Ở hoạt động Luyện tập, GV mở bài tập tương tác phân loại: máy hiện lần lượt các việc nhà, HS chọn việc vừa sức và an toàn hay việc phải nhờ người lớn…
 KNS: KN tự phục vụ: tự làm lấy việc của mình, giữ gìn vệ sinh cá nhân và nơi ở.</t>
         </is>
       </c>
@@ -1657,7 +1664,8 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>NLS-GQVĐ (Cơ bản 1): Nêu và làm mẫu cách người lớn quét mã trên bao bì để tra thông tin sản phẩm.</t>
+          <t>Năng lực số Miền 1 (Cơ bản, bậc 1): GV chiếu ảnh phóng to nhãn một gói bánh, hộp sữa lên màn hình, chỉ cho HS chỗ ghi hạn sử dụng và hướng dẫn HS đọc số ngày tháng ghi ở đó.
+Năng lực số Miền 5 (Cơ bản, bậc 1): GV nêu và làm mẫu cách người lớn quét mã trên bao bì để tra thông tin sản phẩm; HS quan sát GV thao tác và nói lại việc cần làm trước khi ăn…</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Đồng bộ hai website theo app bản 192 (KHGD chữ in hoa → chữ thường)
Chạy _khgd-app-to-web.py cho lớp 1–5 sau khi app đổi 3.629 ô Chủ đề/Tên bài từ chữ
in hoa về chữ thường (giữ tên riêng, viết tắt, số La Mã). Cột 7 lấy từ _cot7-day.json
xuất lại cùng ngày. Đo web-vs-app: 102 lượt môn, 0 dòng lệch ở cả website và web-chung.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ucMYKvcHtg5qiGKrbLvpM
</commit_message>
<xml_diff>
--- a/assets/docs/lop1/Dao duc - Lop 1.xlsx
+++ b/assets/docs/lop1/Dao duc - Lop 1.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>CĐ 1: TỰ CHĂM SÓC</t>
+          <t>CĐ 1: Tự chăm sóc</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
@@ -570,7 +570,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>CĐ 1: TỰ CHĂM SÓC</t>
+          <t>CĐ 1: Tự chăm sóc</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr"/>
@@ -605,7 +605,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>CĐ 1: TỰ CHĂM SÓC</t>
+          <t>CĐ 1: Tự chăm sóc</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
@@ -640,7 +640,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>CĐ 1: TỰ CHĂM SÓC</t>
+          <t>CĐ 1: Tự chăm sóc</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
@@ -676,7 +676,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>CĐ 2: YÊU THƯƠNG</t>
+          <t>CĐ 2: Yêu thương</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
@@ -711,7 +711,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>CĐ 2: YÊU THƯƠNG</t>
+          <t>CĐ 2: Yêu thương</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
@@ -745,7 +745,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>CĐ 3: QUAN TÂM CHĂM SÓC NGƯỜI THÂN TRONG GIA ĐÌNH</t>
+          <t>CĐ 3: Quan tâm chăm sóc người thân trong gia đình</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
@@ -779,7 +779,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>CĐ 3: QUAN TÂM CHĂM SÓC NGƯỜI THÂN TRONG GIA ĐÌNH</t>
+          <t>CĐ 3: Quan tâm chăm sóc người thân trong gia đình</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
@@ -813,7 +813,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>CĐ 3: QUAN TÂM CHĂM SÓC NGƯỜI THÂN TRONG GIA ĐÌNH</t>
+          <t>CĐ 3: Quan tâm chăm sóc người thân trong gia đình</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
@@ -847,7 +847,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>CĐ 3: QUAN TÂM CHĂM SÓC NGƯỜI THÂN TRONG GIA ĐÌNH</t>
+          <t>CĐ 3: Quan tâm chăm sóc người thân trong gia đình</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
@@ -882,7 +882,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>CĐ 3: QUAN TÂM CHĂM SÓC NGƯỜI THÂN TRONG GIA ĐÌNH</t>
+          <t>CĐ 3: Quan tâm chăm sóc người thân trong gia đình</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr"/>
@@ -912,7 +912,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>CĐ4: THỰC HIỆN NỘI QUY TRƯỜNG LỚP</t>
+          <t>CĐ4: Thực hiện nội quy trường lớp</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
@@ -948,7 +948,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>CĐ4: THỰC HIỆN NỘI QUY TRƯỜNG LỚP</t>
+          <t>CĐ4: Thực hiện nội quy trường lớp</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr"/>
@@ -982,7 +982,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>CĐ4: THỰC HIỆN NỘI QUY TRƯỜNG LỚP</t>
+          <t>CĐ4: Thực hiện nội quy trường lớp</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr"/>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>CĐ4: THỰC HIỆN NỘI QUY TRƯỜNG LỚP</t>
+          <t>CĐ4: Thực hiện nội quy trường lớp</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr"/>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>CĐ4: THỰC HIỆN NỘI QUY TRƯỜNG LỚP</t>
+          <t>CĐ4: Thực hiện nội quy trường lớp</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr"/>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>CĐ 5: SINH HOẠT NỀN NẾP</t>
+          <t>CĐ 5: Sinh hoạt nền nếp</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr"/>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>CĐ 5: SINH HOẠT NỀN NẾP</t>
+          <t>CĐ 5: Sinh hoạt nền nếp</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr"/>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>CĐ 5: SINH HOẠT NỀN NẾP</t>
+          <t>CĐ 5: Sinh hoạt nền nếp</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr"/>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>CĐ 6: TỰ GIÁC LÀM VIỆC CỦA MÌNH</t>
+          <t>CĐ 6: Tự giác làm việc của mình</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr"/>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>CĐ 6: TỰ GIÁC LÀM VIỆC CỦA MÌNH</t>
+          <t>CĐ 6: Tự giác làm việc của mình</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr"/>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>CĐ 6: TỰ GIÁC LÀM VIỆC CỦA MÌNH</t>
+          <t>CĐ 6: Tự giác làm việc của mình</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr"/>
@@ -1303,7 +1303,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>CĐ 7: THẬT THÀ</t>
+          <t>CĐ 7: Thật thà</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr"/>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>CĐ 7: THẬT THÀ</t>
+          <t>CĐ 7: Thật thà</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr"/>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>CĐ 7: THẬT THÀ</t>
+          <t>CĐ 7: Thật thà</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr"/>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>CĐ 7: THẬT THÀ</t>
+          <t>CĐ 7: Thật thà</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr"/>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>CĐ 7: THẬT THÀ</t>
+          <t>CĐ 7: Thật thà</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr"/>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>CĐ 8: PHÒNG TRÁNH TAI NẠN, THƯƠNG TÍCH</t>
+          <t>CĐ 8: Phòng tránh tai nạn, thương tích</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr"/>
@@ -1506,7 +1506,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>CĐ 8: PHÒNG TRÁNH TAI NẠN, THƯƠNG TÍCH</t>
+          <t>CĐ 8: Phòng tránh tai nạn, thương tích</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr"/>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>CĐ 8: PHÒNG TRÁNH TAI NẠN, THƯƠNG TÍCH</t>
+          <t>CĐ 8: Phòng tránh tai nạn, thương tích</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr"/>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>CĐ 8: PHÒNG TRÁNH TAI NẠN, THƯƠNG TÍCH</t>
+          <t>CĐ 8: Phòng tránh tai nạn, thương tích</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr"/>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>CĐ 8: PHÒNG TRÁNH TAI NẠN, THƯƠNG TÍCH</t>
+          <t>CĐ 8: Phòng tránh tai nạn, thương tích</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr"/>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>CĐ 8: PHÒNG TRÁNH TAI NẠN, THƯƠNG TÍCH</t>
+          <t>CĐ 8: Phòng tránh tai nạn, thương tích</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr"/>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>CĐ 8: PHÒNG TRÁNH TAI NẠN, THƯƠNG TÍCH</t>
+          <t>CĐ 8: Phòng tránh tai nạn, thương tích</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr"/>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>CĐ 8: PHÒNG TRÁNH TAI NẠN, THƯƠNG TÍCH</t>
+          <t>CĐ 8: Phòng tránh tai nạn, thương tích</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr"/>

</xml_diff>